<commit_message>
Actualizacion de inventario: CARA, ALMACEN e ITEAM
</commit_message>
<xml_diff>
--- a/INVENTARIO LA JOYA ATT OFICIAL.xlsx
+++ b/INVENTARIO LA JOYA ATT OFICIAL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Romario\Documents\Proyecto AT&amp;T\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CED32F6F-0347-4D9B-BD6D-462626315913}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7DFE9DC-4BFA-4240-9C94-E802754C4478}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{78AC62DE-59EB-455E-B97D-A507C5B93E50}"/>
   </bookViews>
@@ -5426,16 +5426,22 @@
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000467</t>
+          <t xml:space="preserve">467</t>
         </is>
       </c>
       <c r="B2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="4"/>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ATRAS</t>
+        </is>
+      </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
+      <c r="F2" s="4" t="s">
+        <v>15</v>
+      </c>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
@@ -5449,7 +5455,7 @@
     <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000001</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="B3" s="4" t="s">
@@ -5490,7 +5496,7 @@
     <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000002</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="B4" s="4" t="s">
@@ -5531,7 +5537,7 @@
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000003</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="B5" s="4" t="s">
@@ -5572,7 +5578,7 @@
     <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000004</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="B6" s="4" t="s">
@@ -5613,7 +5619,7 @@
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000005</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
       <c r="B7" s="4" t="s">
@@ -5654,7 +5660,7 @@
     <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000006</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="B8" s="4" t="s">
@@ -5695,7 +5701,7 @@
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000007</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="B9" s="4" t="s">
@@ -5736,7 +5742,7 @@
     <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000008</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="B10" s="4" t="s">
@@ -5777,7 +5783,7 @@
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000009</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="B11" s="4" t="s">
@@ -5818,7 +5824,7 @@
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000010</t>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
       <c r="B12" s="4" t="s">
@@ -5859,7 +5865,7 @@
     <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000011</t>
+          <t xml:space="preserve">11</t>
         </is>
       </c>
       <c r="B13" s="4" t="s">
@@ -5900,7 +5906,7 @@
     <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000012</t>
+          <t xml:space="preserve">12</t>
         </is>
       </c>
       <c r="B14" s="4" t="s">
@@ -5941,7 +5947,7 @@
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000013</t>
+          <t xml:space="preserve">13</t>
         </is>
       </c>
       <c r="B15" s="4" t="s">
@@ -5982,7 +5988,7 @@
     <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000014</t>
+          <t xml:space="preserve">14</t>
         </is>
       </c>
       <c r="B16" s="4" t="s">
@@ -6023,7 +6029,7 @@
     <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000015</t>
+          <t xml:space="preserve">15</t>
         </is>
       </c>
       <c r="B17" s="4" t="s">
@@ -6064,7 +6070,7 @@
     <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000016</t>
+          <t xml:space="preserve">16</t>
         </is>
       </c>
       <c r="B18" s="4" t="s">
@@ -6105,7 +6111,7 @@
     <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000017</t>
+          <t xml:space="preserve">17</t>
         </is>
       </c>
       <c r="B19" s="4" t="s">
@@ -6146,7 +6152,7 @@
     <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000018</t>
+          <t xml:space="preserve">18</t>
         </is>
       </c>
       <c r="B20" s="4" t="s">
@@ -6187,7 +6193,7 @@
     <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000019</t>
+          <t xml:space="preserve">19</t>
         </is>
       </c>
       <c r="B21" s="4" t="s">
@@ -6228,7 +6234,7 @@
     <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000020</t>
+          <t xml:space="preserve">20</t>
         </is>
       </c>
       <c r="B22" s="4" t="s">
@@ -6269,7 +6275,7 @@
     <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000021</t>
+          <t xml:space="preserve">21</t>
         </is>
       </c>
       <c r="B23" s="4" t="s">
@@ -6310,7 +6316,7 @@
     <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000022</t>
+          <t xml:space="preserve">22</t>
         </is>
       </c>
       <c r="B24" s="4" t="s">
@@ -6351,7 +6357,7 @@
     <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000023</t>
+          <t xml:space="preserve">23</t>
         </is>
       </c>
       <c r="B25" s="4" t="s">
@@ -6390,7 +6396,7 @@
     <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000024</t>
+          <t xml:space="preserve">24</t>
         </is>
       </c>
       <c r="B26" s="4" t="s">
@@ -6431,7 +6437,7 @@
     <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000025</t>
+          <t xml:space="preserve">25</t>
         </is>
       </c>
       <c r="B27" s="4" t="s">
@@ -6472,7 +6478,7 @@
     <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000026</t>
+          <t xml:space="preserve">26</t>
         </is>
       </c>
       <c r="B28" s="4" t="s">
@@ -6513,7 +6519,7 @@
     <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000027</t>
+          <t xml:space="preserve">27</t>
         </is>
       </c>
       <c r="B29" s="4" t="s">
@@ -6554,7 +6560,7 @@
     <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000028</t>
+          <t xml:space="preserve">28</t>
         </is>
       </c>
       <c r="B30" s="4" t="s">
@@ -6595,7 +6601,7 @@
     <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000029</t>
+          <t xml:space="preserve">29</t>
         </is>
       </c>
       <c r="B31" s="4" t="s">
@@ -6636,7 +6642,7 @@
     <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000030</t>
+          <t xml:space="preserve">30</t>
         </is>
       </c>
       <c r="B32" s="4" t="s">
@@ -6677,7 +6683,7 @@
     <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000031</t>
+          <t xml:space="preserve">31</t>
         </is>
       </c>
       <c r="B33" s="4" t="s">
@@ -6718,7 +6724,7 @@
     <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000032</t>
+          <t xml:space="preserve">32</t>
         </is>
       </c>
       <c r="B34" s="4" t="s">
@@ -6759,7 +6765,7 @@
     <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000033</t>
+          <t xml:space="preserve">33</t>
         </is>
       </c>
       <c r="B35" s="4" t="s">
@@ -6800,7 +6806,7 @@
     <row r="36" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000034</t>
+          <t xml:space="preserve">34</t>
         </is>
       </c>
       <c r="B36" s="4" t="s">
@@ -6841,7 +6847,7 @@
     <row r="37" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000035</t>
+          <t xml:space="preserve">35</t>
         </is>
       </c>
       <c r="B37" s="4" t="s">
@@ -6882,7 +6888,7 @@
     <row r="38" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000036</t>
+          <t xml:space="preserve">36</t>
         </is>
       </c>
       <c r="B38" s="4" t="s">
@@ -6923,7 +6929,7 @@
     <row r="39" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000037</t>
+          <t xml:space="preserve">37</t>
         </is>
       </c>
       <c r="B39" s="4" t="s">
@@ -6964,7 +6970,7 @@
     <row r="40" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000038</t>
+          <t xml:space="preserve">38</t>
         </is>
       </c>
       <c r="B40" s="4" t="s">
@@ -7005,7 +7011,7 @@
     <row r="41" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000039</t>
+          <t xml:space="preserve">39</t>
         </is>
       </c>
       <c r="B41" s="4" t="s">
@@ -7046,7 +7052,7 @@
     <row r="42" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000040</t>
+          <t xml:space="preserve">40</t>
         </is>
       </c>
       <c r="B42" s="4" t="s">
@@ -7087,7 +7093,7 @@
     <row r="43" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000041</t>
+          <t xml:space="preserve">41</t>
         </is>
       </c>
       <c r="B43" s="4" t="s">
@@ -7128,7 +7134,7 @@
     <row r="44" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000042</t>
+          <t xml:space="preserve">42</t>
         </is>
       </c>
       <c r="B44" s="4" t="s">
@@ -7169,7 +7175,7 @@
     <row r="45" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000043</t>
+          <t xml:space="preserve">43</t>
         </is>
       </c>
       <c r="B45" s="4" t="s">
@@ -7210,7 +7216,7 @@
     <row r="46" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000044</t>
+          <t xml:space="preserve">44</t>
         </is>
       </c>
       <c r="B46" s="4" t="s">
@@ -7251,7 +7257,7 @@
     <row r="47" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000045</t>
+          <t xml:space="preserve">45</t>
         </is>
       </c>
       <c r="B47" s="4" t="s">
@@ -7292,7 +7298,7 @@
     <row r="48" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000046</t>
+          <t xml:space="preserve">46</t>
         </is>
       </c>
       <c r="B48" s="4" t="s">
@@ -7333,7 +7339,7 @@
     <row r="49" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000047</t>
+          <t xml:space="preserve">47</t>
         </is>
       </c>
       <c r="B49" s="4" t="s">
@@ -7374,7 +7380,7 @@
     <row r="50" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000048</t>
+          <t xml:space="preserve">48</t>
         </is>
       </c>
       <c r="B50" s="4" t="s">
@@ -7415,7 +7421,7 @@
     <row r="51" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000049</t>
+          <t xml:space="preserve">49</t>
         </is>
       </c>
       <c r="B51" s="4" t="s">
@@ -7456,7 +7462,7 @@
     <row r="52" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000050</t>
+          <t xml:space="preserve">50</t>
         </is>
       </c>
       <c r="B52" s="4" t="s">
@@ -7497,7 +7503,7 @@
     <row r="53" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000051</t>
+          <t xml:space="preserve">51</t>
         </is>
       </c>
       <c r="B53" s="4" t="s">
@@ -7561,7 +7567,7 @@
     <row r="55" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000052</t>
+          <t xml:space="preserve">52</t>
         </is>
       </c>
       <c r="B55" s="4" t="s">
@@ -7602,7 +7608,7 @@
     <row r="56" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000053</t>
+          <t xml:space="preserve">53</t>
         </is>
       </c>
       <c r="B56" s="4" t="s">
@@ -7643,7 +7649,7 @@
     <row r="57" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000054</t>
+          <t xml:space="preserve">54</t>
         </is>
       </c>
       <c r="B57" s="4" t="s">
@@ -7684,7 +7690,7 @@
     <row r="58" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000055</t>
+          <t xml:space="preserve">55</t>
         </is>
       </c>
       <c r="B58" s="4" t="s">
@@ -7725,7 +7731,7 @@
     <row r="59" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000056</t>
+          <t xml:space="preserve">56</t>
         </is>
       </c>
       <c r="B59" s="4" t="s">
@@ -7766,7 +7772,7 @@
     <row r="60" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000057</t>
+          <t xml:space="preserve">57</t>
         </is>
       </c>
       <c r="B60" s="4" t="s">
@@ -7807,7 +7813,7 @@
     <row r="61" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000058</t>
+          <t xml:space="preserve">58</t>
         </is>
       </c>
       <c r="B61" s="4" t="s">
@@ -7848,7 +7854,7 @@
     <row r="62" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000059</t>
+          <t xml:space="preserve">59</t>
         </is>
       </c>
       <c r="B62" s="4" t="s">
@@ -7889,7 +7895,7 @@
     <row r="63" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000060</t>
+          <t xml:space="preserve">60</t>
         </is>
       </c>
       <c r="B63" s="4" t="s">
@@ -7930,7 +7936,7 @@
     <row r="64" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000061</t>
+          <t xml:space="preserve">61</t>
         </is>
       </c>
       <c r="B64" s="4" t="s">
@@ -7971,7 +7977,7 @@
     <row r="65" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000062</t>
+          <t xml:space="preserve">62</t>
         </is>
       </c>
       <c r="B65" s="4" t="s">
@@ -8012,7 +8018,7 @@
     <row r="66" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000063</t>
+          <t xml:space="preserve">63</t>
         </is>
       </c>
       <c r="B66" s="4" t="s">
@@ -8051,7 +8057,7 @@
     <row r="67" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000064</t>
+          <t xml:space="preserve">64</t>
         </is>
       </c>
       <c r="B67" s="4" t="s">
@@ -8092,7 +8098,7 @@
     <row r="68" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000065</t>
+          <t xml:space="preserve">65</t>
         </is>
       </c>
       <c r="B68" s="4" t="s">
@@ -8208,7 +8214,7 @@
     <row r="72" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000066</t>
+          <t xml:space="preserve">66</t>
         </is>
       </c>
       <c r="B72" s="4" t="s">
@@ -8249,7 +8255,7 @@
     <row r="73" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000067</t>
+          <t xml:space="preserve">67</t>
         </is>
       </c>
       <c r="B73" s="4" t="s">
@@ -8290,7 +8296,7 @@
     <row r="74" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000068</t>
+          <t xml:space="preserve">68</t>
         </is>
       </c>
       <c r="B74" s="4" t="s">
@@ -8331,7 +8337,7 @@
     <row r="75" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000069</t>
+          <t xml:space="preserve">69</t>
         </is>
       </c>
       <c r="B75" s="4" t="s">
@@ -8372,7 +8378,7 @@
     <row r="76" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000070</t>
+          <t xml:space="preserve">70</t>
         </is>
       </c>
       <c r="B76" s="4" t="s">
@@ -8463,7 +8469,7 @@
     <row r="79" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000071</t>
+          <t xml:space="preserve">71</t>
         </is>
       </c>
       <c r="B79" s="4" t="s">
@@ -8500,7 +8506,7 @@
     <row r="80" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000072</t>
+          <t xml:space="preserve">72</t>
         </is>
       </c>
       <c r="B80" s="4" t="s">
@@ -8539,7 +8545,7 @@
     <row r="81" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000073</t>
+          <t xml:space="preserve">73</t>
         </is>
       </c>
       <c r="B81" s="4" t="s">
@@ -8580,7 +8586,7 @@
     <row r="82" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000074</t>
+          <t xml:space="preserve">74</t>
         </is>
       </c>
       <c r="B82" s="4" t="s">
@@ -8617,7 +8623,7 @@
     <row r="83" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000075</t>
+          <t xml:space="preserve">75</t>
         </is>
       </c>
       <c r="B83" s="4" t="s">
@@ -8658,7 +8664,7 @@
     <row r="84" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000076</t>
+          <t xml:space="preserve">76</t>
         </is>
       </c>
       <c r="B84" s="4" t="s">
@@ -8724,7 +8730,7 @@
     <row r="86" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000077</t>
+          <t xml:space="preserve">77</t>
         </is>
       </c>
       <c r="B86" s="4" t="s">
@@ -8765,7 +8771,7 @@
     <row r="87" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000078</t>
+          <t xml:space="preserve">78</t>
         </is>
       </c>
       <c r="B87" s="4" t="s">
@@ -8806,7 +8812,7 @@
     <row r="88" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000079</t>
+          <t xml:space="preserve">79</t>
         </is>
       </c>
       <c r="B88" s="4" t="s">
@@ -8843,7 +8849,7 @@
     <row r="89" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000080</t>
+          <t xml:space="preserve">80</t>
         </is>
       </c>
       <c r="B89" s="4" t="s">
@@ -8882,7 +8888,7 @@
     <row r="90" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000081</t>
+          <t xml:space="preserve">81</t>
         </is>
       </c>
       <c r="B90" s="4" t="s">
@@ -9023,7 +9029,7 @@
     <row r="95" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000082</t>
+          <t xml:space="preserve">82</t>
         </is>
       </c>
       <c r="B95" s="4" t="s">
@@ -9214,7 +9220,7 @@
     <row r="102" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000083</t>
+          <t xml:space="preserve">83</t>
         </is>
       </c>
       <c r="B102" s="4" t="s">
@@ -9253,7 +9259,7 @@
     <row r="103" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000084</t>
+          <t xml:space="preserve">84</t>
         </is>
       </c>
       <c r="B103" s="4" t="s">
@@ -9294,7 +9300,7 @@
     <row r="104" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000085</t>
+          <t xml:space="preserve">85</t>
         </is>
       </c>
       <c r="B104" s="4" t="s">
@@ -9335,7 +9341,7 @@
     <row r="105" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000086</t>
+          <t xml:space="preserve">86</t>
         </is>
       </c>
       <c r="B105" s="4" t="s">
@@ -9451,7 +9457,7 @@
     <row r="109" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000087</t>
+          <t xml:space="preserve">87</t>
         </is>
       </c>
       <c r="B109" s="4" t="s">
@@ -9490,7 +9496,7 @@
     <row r="110" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000088</t>
+          <t xml:space="preserve">88</t>
         </is>
       </c>
       <c r="B110" s="4" t="s">
@@ -9631,7 +9637,7 @@
     <row r="115" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A115" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000089</t>
+          <t xml:space="preserve">89</t>
         </is>
       </c>
       <c r="B115" s="4" t="s">
@@ -9670,7 +9676,7 @@
     <row r="116" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A116" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000090</t>
+          <t xml:space="preserve">90</t>
         </is>
       </c>
       <c r="B116" s="4" t="s">
@@ -9713,7 +9719,7 @@
     <row r="117" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000091</t>
+          <t xml:space="preserve">91</t>
         </is>
       </c>
       <c r="B117" s="4" t="s">
@@ -9752,7 +9758,7 @@
     <row r="118" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A118" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000092</t>
+          <t xml:space="preserve">92</t>
         </is>
       </c>
       <c r="B118" s="4" t="s">
@@ -9791,7 +9797,7 @@
     <row r="119" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A119" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000093</t>
+          <t xml:space="preserve">93</t>
         </is>
       </c>
       <c r="B119" s="4" t="s">
@@ -9832,7 +9838,7 @@
     <row r="120" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000094</t>
+          <t xml:space="preserve">94</t>
         </is>
       </c>
       <c r="B120" s="4" t="s">
@@ -9871,7 +9877,7 @@
     <row r="121" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A121" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000095</t>
+          <t xml:space="preserve">95</t>
         </is>
       </c>
       <c r="B121" s="4" t="s">
@@ -9912,7 +9918,7 @@
     <row r="122" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A122" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000096</t>
+          <t xml:space="preserve">96</t>
         </is>
       </c>
       <c r="B122" s="4" t="s">
@@ -9953,7 +9959,7 @@
     <row r="123" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A123" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000097</t>
+          <t xml:space="preserve">97</t>
         </is>
       </c>
       <c r="B123" s="4" t="s">
@@ -9994,7 +10000,7 @@
     <row r="124" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A124" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000098</t>
+          <t xml:space="preserve">98</t>
         </is>
       </c>
       <c r="B124" s="4" t="s">
@@ -10035,7 +10041,7 @@
     <row r="125" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A125" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000099</t>
+          <t xml:space="preserve">99</t>
         </is>
       </c>
       <c r="B125" s="4" t="s">
@@ -10076,7 +10082,7 @@
     <row r="126" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A126" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000100</t>
+          <t xml:space="preserve">100</t>
         </is>
       </c>
       <c r="B126" s="4" t="s">
@@ -10117,7 +10123,7 @@
     <row r="127" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A127" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000101</t>
+          <t xml:space="preserve">101</t>
         </is>
       </c>
       <c r="B127" s="4" t="s">
@@ -10158,7 +10164,7 @@
     <row r="128" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A128" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000102</t>
+          <t xml:space="preserve">102</t>
         </is>
       </c>
       <c r="B128" s="4" t="s">
@@ -10199,7 +10205,7 @@
     <row r="129" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A129" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000103</t>
+          <t xml:space="preserve">103</t>
         </is>
       </c>
       <c r="B129" s="4" t="s">
@@ -10240,7 +10246,7 @@
     <row r="130" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A130" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000104</t>
+          <t xml:space="preserve">104</t>
         </is>
       </c>
       <c r="B130" s="4" t="s">
@@ -10281,7 +10287,7 @@
     <row r="131" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A131" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000105</t>
+          <t xml:space="preserve">105</t>
         </is>
       </c>
       <c r="B131" s="4" t="s">
@@ -10322,7 +10328,7 @@
     <row r="132" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A132" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000106</t>
+          <t xml:space="preserve">106</t>
         </is>
       </c>
       <c r="B132" s="4" t="s">
@@ -10438,7 +10444,7 @@
     <row r="136" spans="1:13" s="29" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A136" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000107</t>
+          <t xml:space="preserve">107</t>
         </is>
       </c>
       <c r="B136" s="4" t="s">
@@ -10529,7 +10535,7 @@
     <row r="139" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A139" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000108</t>
+          <t xml:space="preserve">108</t>
         </is>
       </c>
       <c r="B139" s="4" t="s">
@@ -10566,7 +10572,7 @@
     <row r="140" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A140" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000109</t>
+          <t xml:space="preserve">109</t>
         </is>
       </c>
       <c r="B140" s="4" t="s">
@@ -10651,7 +10657,7 @@
     <row r="143" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A143" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000110</t>
+          <t xml:space="preserve">110</t>
         </is>
       </c>
       <c r="B143" s="4" t="s">
@@ -10817,7 +10823,7 @@
     <row r="149" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A149" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000111</t>
+          <t xml:space="preserve">111</t>
         </is>
       </c>
       <c r="B149" s="4" t="s">
@@ -10858,7 +10864,7 @@
     <row r="150" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000112</t>
+          <t xml:space="preserve">112</t>
         </is>
       </c>
       <c r="B150" s="4" t="s">
@@ -10899,7 +10905,7 @@
     <row r="151" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000113</t>
+          <t xml:space="preserve">113</t>
         </is>
       </c>
       <c r="B151" s="4" t="s">
@@ -10942,7 +10948,7 @@
     <row r="152" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A152" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000114</t>
+          <t xml:space="preserve">114</t>
         </is>
       </c>
       <c r="B152" s="4" t="s">
@@ -11010,7 +11016,7 @@
     <row r="154" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000115</t>
+          <t xml:space="preserve">115</t>
         </is>
       </c>
       <c r="B154" s="4" t="s">
@@ -11049,7 +11055,7 @@
     <row r="155" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A155" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000116</t>
+          <t xml:space="preserve">116</t>
         </is>
       </c>
       <c r="B155" s="4" t="s">
@@ -11088,7 +11094,7 @@
     <row r="156" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000117</t>
+          <t xml:space="preserve">117</t>
         </is>
       </c>
       <c r="B156" s="4" t="s">
@@ -11123,7 +11129,7 @@
     <row r="157" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A157" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000118</t>
+          <t xml:space="preserve">118</t>
         </is>
       </c>
       <c r="B157" s="4" t="s">
@@ -11164,7 +11170,7 @@
     <row r="158" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000119</t>
+          <t xml:space="preserve">119</t>
         </is>
       </c>
       <c r="B158" s="4" t="s">
@@ -11255,7 +11261,7 @@
     <row r="161" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000120</t>
+          <t xml:space="preserve">120</t>
         </is>
       </c>
       <c r="B161" s="4" t="s">
@@ -11344,7 +11350,7 @@
     <row r="164" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A164" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000121</t>
+          <t xml:space="preserve">121</t>
         </is>
       </c>
       <c r="B164" s="4" t="s">
@@ -11385,7 +11391,7 @@
     <row r="165" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A165" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000122</t>
+          <t xml:space="preserve">122</t>
         </is>
       </c>
       <c r="B165" s="4" t="s">
@@ -11426,7 +11432,7 @@
     <row r="166" spans="1:13" s="31" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A166" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000123</t>
+          <t xml:space="preserve">123</t>
         </is>
       </c>
       <c r="B166" s="30" t="s">
@@ -11492,7 +11498,7 @@
     <row r="168" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000124</t>
+          <t xml:space="preserve">124</t>
         </is>
       </c>
       <c r="B168" s="4" t="s">
@@ -11658,7 +11664,7 @@
     <row r="174" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000125</t>
+          <t xml:space="preserve">125</t>
         </is>
       </c>
       <c r="B174" s="4" t="s">
@@ -11695,7 +11701,7 @@
     <row r="175" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000126</t>
+          <t xml:space="preserve">126</t>
         </is>
       </c>
       <c r="B175" s="4" t="s">
@@ -11736,7 +11742,7 @@
     <row r="176" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A176" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000127</t>
+          <t xml:space="preserve">127</t>
         </is>
       </c>
       <c r="B176" s="4" t="s">
@@ -11852,7 +11858,7 @@
     <row r="180" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A180" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000128</t>
+          <t xml:space="preserve">128</t>
         </is>
       </c>
       <c r="B180" s="4" t="s">
@@ -11893,7 +11899,7 @@
     <row r="181" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000129</t>
+          <t xml:space="preserve">129</t>
         </is>
       </c>
       <c r="B181" s="4" t="s">
@@ -11957,7 +11963,7 @@
     <row r="183" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000130</t>
+          <t xml:space="preserve">130</t>
         </is>
       </c>
       <c r="B183" s="4" t="s">
@@ -11998,7 +12004,7 @@
     <row r="184" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A184" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000131</t>
+          <t xml:space="preserve">131</t>
         </is>
       </c>
       <c r="B184" s="4" t="s">
@@ -12064,7 +12070,7 @@
     <row r="186" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000132</t>
+          <t xml:space="preserve">132</t>
         </is>
       </c>
       <c r="B186" s="4" t="s">
@@ -12103,7 +12109,7 @@
     <row r="187" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000133</t>
+          <t xml:space="preserve">133</t>
         </is>
       </c>
       <c r="B187" s="4" t="s">
@@ -12169,7 +12175,7 @@
     <row r="189" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A189" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000134</t>
+          <t xml:space="preserve">134</t>
         </is>
       </c>
       <c r="B189" s="4" t="s">
@@ -12208,7 +12214,7 @@
     <row r="190" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000135</t>
+          <t xml:space="preserve">135</t>
         </is>
       </c>
       <c r="B190" s="4" t="s">
@@ -12247,7 +12253,7 @@
     <row r="191" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000136</t>
+          <t xml:space="preserve">136</t>
         </is>
       </c>
       <c r="B191" s="4" t="s">
@@ -12288,7 +12294,7 @@
     <row r="192" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000137</t>
+          <t xml:space="preserve">137</t>
         </is>
       </c>
       <c r="B192" s="4" t="s">
@@ -12329,7 +12335,7 @@
     <row r="193" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000138</t>
+          <t xml:space="preserve">138</t>
         </is>
       </c>
       <c r="B193" s="4" t="s">
@@ -12370,7 +12376,7 @@
     <row r="194" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A194" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000139</t>
+          <t xml:space="preserve">139</t>
         </is>
       </c>
       <c r="B194" s="4" t="s">
@@ -12463,7 +12469,7 @@
     <row r="197" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000140</t>
+          <t xml:space="preserve">140</t>
         </is>
       </c>
       <c r="B197" s="4" t="s">
@@ -12552,7 +12558,7 @@
     <row r="200" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A200" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000141</t>
+          <t xml:space="preserve">141</t>
         </is>
       </c>
       <c r="B200" s="4" t="s">
@@ -12593,7 +12599,7 @@
     <row r="201" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A201" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000142</t>
+          <t xml:space="preserve">142</t>
         </is>
       </c>
       <c r="B201" s="4" t="s">
@@ -12653,7 +12659,7 @@
     <row r="203" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000143</t>
+          <t xml:space="preserve">143</t>
         </is>
       </c>
       <c r="B203" s="4" t="s">
@@ -12769,7 +12775,7 @@
     <row r="207" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A207" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000144</t>
+          <t xml:space="preserve">144</t>
         </is>
       </c>
       <c r="B207" s="4" t="s">
@@ -12835,7 +12841,7 @@
     <row r="209" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A209" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000145</t>
+          <t xml:space="preserve">145</t>
         </is>
       </c>
       <c r="B209" s="4" t="s">
@@ -12876,7 +12882,7 @@
     <row r="210" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A210" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000146</t>
+          <t xml:space="preserve">146</t>
         </is>
       </c>
       <c r="B210" s="4" t="s">
@@ -12917,7 +12923,7 @@
     <row r="211" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A211" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000147</t>
+          <t xml:space="preserve">147</t>
         </is>
       </c>
       <c r="B211" s="4" t="s">
@@ -12956,7 +12962,7 @@
     <row r="212" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A212" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000148</t>
+          <t xml:space="preserve">148</t>
         </is>
       </c>
       <c r="B212" s="4" t="s">
@@ -12993,7 +12999,7 @@
     <row r="213" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A213" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000149</t>
+          <t xml:space="preserve">149</t>
         </is>
       </c>
       <c r="B213" s="4" t="s">
@@ -13049,7 +13055,7 @@
     <row r="215" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A215" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000150</t>
+          <t xml:space="preserve">150</t>
         </is>
       </c>
       <c r="B215" s="4" t="s">
@@ -13090,7 +13096,7 @@
     <row r="216" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A216" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000151</t>
+          <t xml:space="preserve">151</t>
         </is>
       </c>
       <c r="B216" s="4" t="s">
@@ -13127,7 +13133,7 @@
     <row r="217" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A217" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000152</t>
+          <t xml:space="preserve">152</t>
         </is>
       </c>
       <c r="B217" s="4" t="s">
@@ -13193,7 +13199,7 @@
     <row r="219" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A219" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000153</t>
+          <t xml:space="preserve">153</t>
         </is>
       </c>
       <c r="B219" s="4" t="s">
@@ -13234,7 +13240,7 @@
     <row r="220" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A220" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000154</t>
+          <t xml:space="preserve">154</t>
         </is>
       </c>
       <c r="B220" s="4" t="s">
@@ -13275,7 +13281,7 @@
     <row r="221" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A221" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000155</t>
+          <t xml:space="preserve">155</t>
         </is>
       </c>
       <c r="B221" s="4" t="s">
@@ -13312,7 +13318,7 @@
     <row r="222" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A222" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000156</t>
+          <t xml:space="preserve">156</t>
         </is>
       </c>
       <c r="B222" s="4" t="s">
@@ -13353,7 +13359,7 @@
     <row r="223" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A223" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000157</t>
+          <t xml:space="preserve">157</t>
         </is>
       </c>
       <c r="B223" s="4" t="s">
@@ -13394,7 +13400,7 @@
     <row r="224" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A224" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000158</t>
+          <t xml:space="preserve">158</t>
         </is>
       </c>
       <c r="B224" s="4" t="s">
@@ -13435,7 +13441,7 @@
     <row r="225" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A225" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000159</t>
+          <t xml:space="preserve">159</t>
         </is>
       </c>
       <c r="B225" s="4" t="s">
@@ -13478,7 +13484,7 @@
     <row r="226" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A226" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000160</t>
+          <t xml:space="preserve">160</t>
         </is>
       </c>
       <c r="B226" s="4" t="s">
@@ -13544,7 +13550,7 @@
     <row r="228" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A228" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000161</t>
+          <t xml:space="preserve">161</t>
         </is>
       </c>
       <c r="B228" s="4" t="s">
@@ -13610,7 +13616,7 @@
     <row r="230" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A230" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000162</t>
+          <t xml:space="preserve">162</t>
         </is>
       </c>
       <c r="B230" s="4" t="s">
@@ -13726,7 +13732,7 @@
     <row r="234" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A234" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000163</t>
+          <t xml:space="preserve">163</t>
         </is>
       </c>
       <c r="B234" s="4" t="s">
@@ -13790,7 +13796,7 @@
     <row r="236" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A236" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000164</t>
+          <t xml:space="preserve">164</t>
         </is>
       </c>
       <c r="B236" s="4" t="s">
@@ -13879,7 +13885,7 @@
     <row r="239" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A239" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000165</t>
+          <t xml:space="preserve">165</t>
         </is>
       </c>
       <c r="B239" s="4" t="s">
@@ -13939,7 +13945,7 @@
     <row r="241" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A241" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000166</t>
+          <t xml:space="preserve">166</t>
         </is>
       </c>
       <c r="B241" s="4" t="s">
@@ -14005,7 +14011,7 @@
     <row r="243" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A243" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000167</t>
+          <t xml:space="preserve">167</t>
         </is>
       </c>
       <c r="B243" s="4" t="s">
@@ -14069,7 +14075,7 @@
     <row r="245" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A245" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000168</t>
+          <t xml:space="preserve">168</t>
         </is>
       </c>
       <c r="B245" s="4" t="s">
@@ -14206,7 +14212,7 @@
     <row r="250" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A250" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000169</t>
+          <t xml:space="preserve">169</t>
         </is>
       </c>
       <c r="B250" s="4" t="s">
@@ -14322,7 +14328,7 @@
     <row r="254" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A254" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000170</t>
+          <t xml:space="preserve">170</t>
         </is>
       </c>
       <c r="B254" s="4" t="s">
@@ -14361,7 +14367,7 @@
     <row r="255" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A255" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000171</t>
+          <t xml:space="preserve">171</t>
         </is>
       </c>
       <c r="B255" s="4" t="s">
@@ -14404,7 +14410,7 @@
     <row r="256" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A256" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000172</t>
+          <t xml:space="preserve">172</t>
         </is>
       </c>
       <c r="B256" s="4" t="s">
@@ -14520,7 +14526,7 @@
     <row r="260" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A260" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000173</t>
+          <t xml:space="preserve">173</t>
         </is>
       </c>
       <c r="B260" s="4" t="s">
@@ -14561,7 +14567,7 @@
     <row r="261" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A261" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000174</t>
+          <t xml:space="preserve">174</t>
         </is>
       </c>
       <c r="B261" s="4" t="s">
@@ -14627,7 +14633,7 @@
     <row r="263" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A263" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000175</t>
+          <t xml:space="preserve">175</t>
         </is>
       </c>
       <c r="B263" s="4" t="s">
@@ -14668,7 +14674,7 @@
     <row r="264" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A264" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000176</t>
+          <t xml:space="preserve">176</t>
         </is>
       </c>
       <c r="B264" s="4" t="s">
@@ -14707,7 +14713,7 @@
     <row r="265" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A265" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000177</t>
+          <t xml:space="preserve">177</t>
         </is>
       </c>
       <c r="B265" s="4" t="s">
@@ -14750,7 +14756,7 @@
     <row r="266" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A266" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000178</t>
+          <t xml:space="preserve">178</t>
         </is>
       </c>
       <c r="B266" s="4" t="s">
@@ -14814,7 +14820,7 @@
     <row r="268" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A268" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000179</t>
+          <t xml:space="preserve">179</t>
         </is>
       </c>
       <c r="B268" s="4" t="s">
@@ -14955,7 +14961,7 @@
     <row r="273" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A273" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000180</t>
+          <t xml:space="preserve">180</t>
         </is>
       </c>
       <c r="B273" s="4" t="s">
@@ -15071,7 +15077,7 @@
     <row r="277" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A277" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000181</t>
+          <t xml:space="preserve">181</t>
         </is>
       </c>
       <c r="B277" s="4" t="s">
@@ -15110,7 +15116,7 @@
     <row r="278" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A278" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000182</t>
+          <t xml:space="preserve">182</t>
         </is>
       </c>
       <c r="B278" s="4" t="s">
@@ -15151,7 +15157,7 @@
     <row r="279" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A279" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000183</t>
+          <t xml:space="preserve">183</t>
         </is>
       </c>
       <c r="B279" s="4" t="s">
@@ -15190,7 +15196,7 @@
     <row r="280" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A280" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000184</t>
+          <t xml:space="preserve">184</t>
         </is>
       </c>
       <c r="B280" s="4" t="s">
@@ -15306,7 +15312,7 @@
     <row r="284" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A284" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000185</t>
+          <t xml:space="preserve">185</t>
         </is>
       </c>
       <c r="B284" s="4" t="s">
@@ -15347,7 +15353,7 @@
     <row r="285" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A285" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000186</t>
+          <t xml:space="preserve">186</t>
         </is>
       </c>
       <c r="B285" s="4" t="s">
@@ -15388,7 +15394,7 @@
     <row r="286" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A286" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000187</t>
+          <t xml:space="preserve">187</t>
         </is>
       </c>
       <c r="B286" s="4" t="s">
@@ -15429,7 +15435,7 @@
     <row r="287" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A287" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000188</t>
+          <t xml:space="preserve">188</t>
         </is>
       </c>
       <c r="B287" s="4" t="s">
@@ -15468,7 +15474,7 @@
     <row r="288" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A288" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000189</t>
+          <t xml:space="preserve">189</t>
         </is>
       </c>
       <c r="B288" s="4" t="s">
@@ -15507,7 +15513,7 @@
     <row r="289" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A289" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000190</t>
+          <t xml:space="preserve">190</t>
         </is>
       </c>
       <c r="B289" s="4" t="s">
@@ -15546,7 +15552,7 @@
     <row r="290" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A290" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000191</t>
+          <t xml:space="preserve">191</t>
         </is>
       </c>
       <c r="B290" s="4" t="s">
@@ -15712,7 +15718,7 @@
     <row r="296" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A296" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000192</t>
+          <t xml:space="preserve">192</t>
         </is>
       </c>
       <c r="B296" s="4" t="s">
@@ -15776,7 +15782,7 @@
     <row r="298" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A298" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000193</t>
+          <t xml:space="preserve">193</t>
         </is>
       </c>
       <c r="B298" s="4" t="s">
@@ -15817,7 +15823,7 @@
     <row r="299" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A299" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000194</t>
+          <t xml:space="preserve">194</t>
         </is>
       </c>
       <c r="B299" s="4" t="s">
@@ -15856,7 +15862,7 @@
     <row r="300" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A300" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000195</t>
+          <t xml:space="preserve">195</t>
         </is>
       </c>
       <c r="B300" s="4" t="s">
@@ -15922,7 +15928,7 @@
     <row r="302" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A302" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000196</t>
+          <t xml:space="preserve">196</t>
         </is>
       </c>
       <c r="B302" s="4" t="s">
@@ -16040,7 +16046,7 @@
     <row r="306" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A306" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000197</t>
+          <t xml:space="preserve">197</t>
         </is>
       </c>
       <c r="B306" s="4" t="s">
@@ -16081,7 +16087,7 @@
     <row r="307" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A307" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000198</t>
+          <t xml:space="preserve">198</t>
         </is>
       </c>
       <c r="B307" s="4" t="s">
@@ -16147,7 +16153,7 @@
     <row r="309" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A309" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000199</t>
+          <t xml:space="preserve">199</t>
         </is>
       </c>
       <c r="B309" s="4" t="s">
@@ -16263,7 +16269,7 @@
     <row r="313" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A313" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000200</t>
+          <t xml:space="preserve">200</t>
         </is>
       </c>
       <c r="B313" s="4" t="s">
@@ -16329,7 +16335,7 @@
     <row r="315" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A315" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000201</t>
+          <t xml:space="preserve">201</t>
         </is>
       </c>
       <c r="B315" s="4" t="s">
@@ -16370,7 +16376,7 @@
     <row r="316" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A316" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000202</t>
+          <t xml:space="preserve">202</t>
         </is>
       </c>
       <c r="B316" s="4" t="s">
@@ -16486,7 +16492,7 @@
     <row r="320" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A320" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000203</t>
+          <t xml:space="preserve">203</t>
         </is>
       </c>
       <c r="B320" s="4" t="s">
@@ -16527,7 +16533,7 @@
     <row r="321" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A321" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000204</t>
+          <t xml:space="preserve">204</t>
         </is>
       </c>
       <c r="B321" s="4" t="s">
@@ -16568,7 +16574,7 @@
     <row r="322" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A322" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000205</t>
+          <t xml:space="preserve">205</t>
         </is>
       </c>
       <c r="B322" s="4" t="s">
@@ -16609,7 +16615,7 @@
     <row r="323" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A323" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000206</t>
+          <t xml:space="preserve">206</t>
         </is>
       </c>
       <c r="B323" s="4" t="s">
@@ -16650,7 +16656,7 @@
     <row r="324" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A324" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000207</t>
+          <t xml:space="preserve">207</t>
         </is>
       </c>
       <c r="B324" s="4" t="s">
@@ -16689,7 +16695,7 @@
     <row r="325" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A325" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000208</t>
+          <t xml:space="preserve">208</t>
         </is>
       </c>
       <c r="B325" s="4" t="s">
@@ -16730,7 +16736,7 @@
     <row r="326" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A326" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000209</t>
+          <t xml:space="preserve">209</t>
         </is>
       </c>
       <c r="B326" s="4" t="s">
@@ -16796,7 +16802,7 @@
     <row r="328" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A328" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000210</t>
+          <t xml:space="preserve">210</t>
         </is>
       </c>
       <c r="B328" s="4" t="s">
@@ -16887,7 +16893,7 @@
     <row r="331" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A331" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000211</t>
+          <t xml:space="preserve">211</t>
         </is>
       </c>
       <c r="B331" s="4" t="s">
@@ -16928,7 +16934,7 @@
     <row r="332" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A332" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000212</t>
+          <t xml:space="preserve">212</t>
         </is>
       </c>
       <c r="B332" s="4" t="s">
@@ -16994,7 +17000,7 @@
     <row r="334" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A334" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000213</t>
+          <t xml:space="preserve">213</t>
         </is>
       </c>
       <c r="B334" s="4" t="s">
@@ -17062,7 +17068,7 @@
     <row r="336" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A336" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000214</t>
+          <t xml:space="preserve">214</t>
         </is>
       </c>
       <c r="B336" s="4" t="s">
@@ -17153,7 +17159,7 @@
     <row r="339" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A339" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000215</t>
+          <t xml:space="preserve">215</t>
         </is>
       </c>
       <c r="B339" s="4" t="s">
@@ -17194,7 +17200,7 @@
     <row r="340" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A340" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000216</t>
+          <t xml:space="preserve">216</t>
         </is>
       </c>
       <c r="B340" s="4" t="s">
@@ -17235,7 +17241,7 @@
     <row r="341" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A341" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000217</t>
+          <t xml:space="preserve">217</t>
         </is>
       </c>
       <c r="B341" s="4" t="s">
@@ -17276,7 +17282,7 @@
     <row r="342" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A342" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000218</t>
+          <t xml:space="preserve">218</t>
         </is>
       </c>
       <c r="B342" s="4" t="s">
@@ -17311,7 +17317,7 @@
     <row r="343" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A343" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000219</t>
+          <t xml:space="preserve">219</t>
         </is>
       </c>
       <c r="B343" s="4" t="s">
@@ -17352,7 +17358,7 @@
     <row r="344" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A344" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000220</t>
+          <t xml:space="preserve">220</t>
         </is>
       </c>
       <c r="B344" s="4" t="s">
@@ -17391,7 +17397,7 @@
     <row r="345" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A345" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000221</t>
+          <t xml:space="preserve">221</t>
         </is>
       </c>
       <c r="B345" s="4" t="s">
@@ -17432,7 +17438,7 @@
     <row r="346" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A346" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000222</t>
+          <t xml:space="preserve">222</t>
         </is>
       </c>
       <c r="B346" s="4" t="s">
@@ -17496,7 +17502,7 @@
     <row r="348" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A348" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000223</t>
+          <t xml:space="preserve">223</t>
         </is>
       </c>
       <c r="B348" s="4" t="s">
@@ -17535,7 +17541,7 @@
     <row r="349" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A349" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000224</t>
+          <t xml:space="preserve">224</t>
         </is>
       </c>
       <c r="B349" s="4" t="s">
@@ -17576,7 +17582,7 @@
     <row r="350" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A350" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000225</t>
+          <t xml:space="preserve">225</t>
         </is>
       </c>
       <c r="B350" s="4" t="s">
@@ -17617,7 +17623,7 @@
     <row r="351" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A351" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000226</t>
+          <t xml:space="preserve">226</t>
         </is>
       </c>
       <c r="B351" s="4" t="s">
@@ -17658,7 +17664,7 @@
     <row r="352" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A352" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000227</t>
+          <t xml:space="preserve">227</t>
         </is>
       </c>
       <c r="B352" s="4" t="s">
@@ -17699,7 +17705,7 @@
     <row r="353" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A353" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000228</t>
+          <t xml:space="preserve">228</t>
         </is>
       </c>
       <c r="B353" s="4" t="s">
@@ -17740,7 +17746,7 @@
     <row r="354" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A354" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000229</t>
+          <t xml:space="preserve">229</t>
         </is>
       </c>
       <c r="B354" s="4" t="s">
@@ -17777,7 +17783,7 @@
     <row r="355" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A355" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000230</t>
+          <t xml:space="preserve">230</t>
         </is>
       </c>
       <c r="B355" s="4" t="s">
@@ -17845,7 +17851,7 @@
     <row r="357" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A357" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000231</t>
+          <t xml:space="preserve">231</t>
         </is>
       </c>
       <c r="B357" s="4" t="s">
@@ -17886,7 +17892,7 @@
     <row r="358" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A358" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000232</t>
+          <t xml:space="preserve">232</t>
         </is>
       </c>
       <c r="B358" s="4" t="s">
@@ -17927,7 +17933,7 @@
     <row r="359" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A359" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000233</t>
+          <t xml:space="preserve">233</t>
         </is>
       </c>
       <c r="B359" s="4" t="s">
@@ -17991,7 +17997,7 @@
     <row r="361" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A361" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000234</t>
+          <t xml:space="preserve">234</t>
         </is>
       </c>
       <c r="B361" s="4" t="s">
@@ -18032,7 +18038,7 @@
     <row r="362" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A362" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000235</t>
+          <t xml:space="preserve">235</t>
         </is>
       </c>
       <c r="B362" s="4" t="s">
@@ -18071,7 +18077,7 @@
     <row r="363" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A363" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000236</t>
+          <t xml:space="preserve">236</t>
         </is>
       </c>
       <c r="B363" s="4" t="s">
@@ -18112,7 +18118,7 @@
     <row r="364" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A364" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000237</t>
+          <t xml:space="preserve">237</t>
         </is>
       </c>
       <c r="B364" s="4" t="s">
@@ -18226,7 +18232,7 @@
     <row r="368" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A368" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000238</t>
+          <t xml:space="preserve">238</t>
         </is>
       </c>
       <c r="B368" s="4" t="s">
@@ -18315,7 +18321,7 @@
     <row r="371" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A371" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000239</t>
+          <t xml:space="preserve">239</t>
         </is>
       </c>
       <c r="B371" s="4" t="s">
@@ -18354,7 +18360,7 @@
     <row r="372" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A372" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000240</t>
+          <t xml:space="preserve">240</t>
         </is>
       </c>
       <c r="B372" s="4" t="s">
@@ -18395,7 +18401,7 @@
     <row r="373" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A373" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000241</t>
+          <t xml:space="preserve">241</t>
         </is>
       </c>
       <c r="B373" s="4" t="s">
@@ -18436,7 +18442,7 @@
     <row r="374" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A374" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000242</t>
+          <t xml:space="preserve">242</t>
         </is>
       </c>
       <c r="B374" s="4" t="s">
@@ -18602,7 +18608,7 @@
     <row r="380" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A380" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000243</t>
+          <t xml:space="preserve">243</t>
         </is>
       </c>
       <c r="B380" s="4" t="s">
@@ -18643,7 +18649,7 @@
     <row r="381" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A381" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000244</t>
+          <t xml:space="preserve">244</t>
         </is>
       </c>
       <c r="B381" s="4" t="s">
@@ -18684,7 +18690,7 @@
     <row r="382" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A382" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000245</t>
+          <t xml:space="preserve">245</t>
         </is>
       </c>
       <c r="B382" s="4" t="s">
@@ -18725,7 +18731,7 @@
     <row r="383" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A383" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000246</t>
+          <t xml:space="preserve">246</t>
         </is>
       </c>
       <c r="B383" s="4" t="s">
@@ -18766,7 +18772,7 @@
     <row r="384" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A384" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000247</t>
+          <t xml:space="preserve">247</t>
         </is>
       </c>
       <c r="B384" s="4" t="s">
@@ -18830,7 +18836,7 @@
     <row r="386" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A386" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000248</t>
+          <t xml:space="preserve">248</t>
         </is>
       </c>
       <c r="B386" s="4" t="s">
@@ -18915,7 +18921,7 @@
     <row r="389" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A389" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000249</t>
+          <t xml:space="preserve">249</t>
         </is>
       </c>
       <c r="B389" s="4" t="s">
@@ -18956,7 +18962,7 @@
     <row r="390" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A390" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000250</t>
+          <t xml:space="preserve">250</t>
         </is>
       </c>
       <c r="B390" s="4" t="s">
@@ -18997,7 +19003,7 @@
     <row r="391" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A391" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000251</t>
+          <t xml:space="preserve">251</t>
         </is>
       </c>
       <c r="B391" s="4" t="s">
@@ -19036,7 +19042,7 @@
     <row r="392" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A392" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000252</t>
+          <t xml:space="preserve">252</t>
         </is>
       </c>
       <c r="B392" s="4" t="s">
@@ -19077,7 +19083,7 @@
     <row r="393" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A393" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000253</t>
+          <t xml:space="preserve">253</t>
         </is>
       </c>
       <c r="B393" s="4" t="s">
@@ -19170,7 +19176,7 @@
     <row r="396" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A396" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000254</t>
+          <t xml:space="preserve">254</t>
         </is>
       </c>
       <c r="B396" s="4" t="s">
@@ -19211,7 +19217,7 @@
     <row r="397" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A397" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000255</t>
+          <t xml:space="preserve">255</t>
         </is>
       </c>
       <c r="B397" s="4" t="s">
@@ -19250,7 +19256,7 @@
     <row r="398" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A398" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000256</t>
+          <t xml:space="preserve">256</t>
         </is>
       </c>
       <c r="B398" s="4" t="s">
@@ -19291,7 +19297,7 @@
     <row r="399" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A399" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000257</t>
+          <t xml:space="preserve">257</t>
         </is>
       </c>
       <c r="B399" s="4" t="s">
@@ -19332,7 +19338,7 @@
     <row r="400" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A400" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000258</t>
+          <t xml:space="preserve">258</t>
         </is>
       </c>
       <c r="B400" s="4" t="s">
@@ -19398,7 +19404,7 @@
     <row r="402" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A402" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000259</t>
+          <t xml:space="preserve">259</t>
         </is>
       </c>
       <c r="B402" s="4" t="s">
@@ -19464,7 +19470,7 @@
     <row r="404" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A404" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000260</t>
+          <t xml:space="preserve">260</t>
         </is>
       </c>
       <c r="B404" s="4" t="s">
@@ -19532,7 +19538,7 @@
     <row r="406" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A406" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000261</t>
+          <t xml:space="preserve">261</t>
         </is>
       </c>
       <c r="B406" s="4" t="s">
@@ -19623,7 +19629,7 @@
     <row r="409" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A409" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000262</t>
+          <t xml:space="preserve">262</t>
         </is>
       </c>
       <c r="B409" s="4" t="s">
@@ -19664,7 +19670,7 @@
     <row r="410" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A410" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000263</t>
+          <t xml:space="preserve">263</t>
         </is>
       </c>
       <c r="B410" s="4" t="s">
@@ -19705,7 +19711,7 @@
     <row r="411" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A411" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000264</t>
+          <t xml:space="preserve">264</t>
         </is>
       </c>
       <c r="B411" s="4" t="s">
@@ -19771,7 +19777,7 @@
     <row r="413" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A413" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000265</t>
+          <t xml:space="preserve">265</t>
         </is>
       </c>
       <c r="B413" s="4" t="s">
@@ -19812,7 +19818,7 @@
     <row r="414" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A414" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000266</t>
+          <t xml:space="preserve">266</t>
         </is>
       </c>
       <c r="B414" s="4" t="s">
@@ -19878,7 +19884,7 @@
     <row r="416" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A416" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000267</t>
+          <t xml:space="preserve">267</t>
         </is>
       </c>
       <c r="B416" s="4" t="s">
@@ -19919,7 +19925,7 @@
     <row r="417" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A417" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000268</t>
+          <t xml:space="preserve">268</t>
         </is>
       </c>
       <c r="B417" s="4" t="s">
@@ -19979,7 +19985,7 @@
     <row r="419" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A419" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000269</t>
+          <t xml:space="preserve">269</t>
         </is>
       </c>
       <c r="B419" s="4" t="s">
@@ -20022,7 +20028,7 @@
     <row r="420" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A420" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000270</t>
+          <t xml:space="preserve">270</t>
         </is>
       </c>
       <c r="B420" s="4" t="s">
@@ -20065,7 +20071,7 @@
     <row r="421" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A421" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000271</t>
+          <t xml:space="preserve">271</t>
         </is>
       </c>
       <c r="B421" s="4" t="s">
@@ -20104,7 +20110,7 @@
     <row r="422" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A422" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000272</t>
+          <t xml:space="preserve">272</t>
         </is>
       </c>
       <c r="B422" s="4" t="s">
@@ -20143,7 +20149,7 @@
     <row r="423" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A423" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000273</t>
+          <t xml:space="preserve">273</t>
         </is>
       </c>
       <c r="B423" s="4" t="s">
@@ -20186,7 +20192,7 @@
     <row r="424" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A424" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000274</t>
+          <t xml:space="preserve">274</t>
         </is>
       </c>
       <c r="B424" s="4" t="s">
@@ -20227,7 +20233,7 @@
     <row r="425" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A425" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000275</t>
+          <t xml:space="preserve">275</t>
         </is>
       </c>
       <c r="B425" s="4" t="s">
@@ -20268,7 +20274,7 @@
     <row r="426" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A426" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000276</t>
+          <t xml:space="preserve">276</t>
         </is>
       </c>
       <c r="B426" s="4" t="s">
@@ -20309,7 +20315,7 @@
     <row r="427" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A427" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000277</t>
+          <t xml:space="preserve">277</t>
         </is>
       </c>
       <c r="B427" s="4" t="s">
@@ -20369,7 +20375,7 @@
     <row r="429" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A429" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000278</t>
+          <t xml:space="preserve">278</t>
         </is>
       </c>
       <c r="B429" s="4" t="s">
@@ -20435,7 +20441,7 @@
     <row r="431" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A431" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000279</t>
+          <t xml:space="preserve">279</t>
         </is>
       </c>
       <c r="B431" s="4" t="s">
@@ -20524,7 +20530,7 @@
     <row r="434" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A434" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000280</t>
+          <t xml:space="preserve">280</t>
         </is>
       </c>
       <c r="B434" s="4" t="s">
@@ -20565,7 +20571,7 @@
     <row r="435" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A435" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000281</t>
+          <t xml:space="preserve">281</t>
         </is>
       </c>
       <c r="B435" s="4" t="s">
@@ -20606,7 +20612,7 @@
     <row r="436" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A436" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000282</t>
+          <t xml:space="preserve">282</t>
         </is>
       </c>
       <c r="B436" s="4" t="s">
@@ -20722,7 +20728,7 @@
     <row r="440" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A440" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000283</t>
+          <t xml:space="preserve">283</t>
         </is>
       </c>
       <c r="B440" s="4" t="s">
@@ -20763,7 +20769,7 @@
     <row r="441" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A441" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000284</t>
+          <t xml:space="preserve">284</t>
         </is>
       </c>
       <c r="B441" s="4" t="s">
@@ -20879,7 +20885,7 @@
     <row r="445" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A445" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000285</t>
+          <t xml:space="preserve">285</t>
         </is>
       </c>
       <c r="B445" s="4" t="s">
@@ -20920,7 +20926,7 @@
     <row r="446" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A446" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000286</t>
+          <t xml:space="preserve">286</t>
         </is>
       </c>
       <c r="B446" s="4" t="s">
@@ -21011,7 +21017,7 @@
     <row r="449" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A449" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000287</t>
+          <t xml:space="preserve">287</t>
         </is>
       </c>
       <c r="B449" s="4" t="s">
@@ -21077,7 +21083,7 @@
     <row r="451" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A451" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000288</t>
+          <t xml:space="preserve">288</t>
         </is>
       </c>
       <c r="B451" s="4" t="s">
@@ -21118,7 +21124,7 @@
     <row r="452" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A452" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000289</t>
+          <t xml:space="preserve">289</t>
         </is>
       </c>
       <c r="B452" s="4" t="s">
@@ -21159,7 +21165,7 @@
     <row r="453" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A453" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000290</t>
+          <t xml:space="preserve">290</t>
         </is>
       </c>
       <c r="B453" s="4" t="s">
@@ -21200,7 +21206,7 @@
     <row r="454" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A454" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000291</t>
+          <t xml:space="preserve">291</t>
         </is>
       </c>
       <c r="B454" s="4" t="s">
@@ -21241,7 +21247,7 @@
     <row r="455" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A455" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000292</t>
+          <t xml:space="preserve">292</t>
         </is>
       </c>
       <c r="B455" s="4" t="s">
@@ -21282,7 +21288,7 @@
     <row r="456" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A456" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000293</t>
+          <t xml:space="preserve">293</t>
         </is>
       </c>
       <c r="B456" s="4" t="s">
@@ -21325,7 +21331,7 @@
     <row r="457" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A457" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000294</t>
+          <t xml:space="preserve">294</t>
         </is>
       </c>
       <c r="B457" s="4" t="s">
@@ -21441,7 +21447,7 @@
     <row r="461" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A461" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000295</t>
+          <t xml:space="preserve">295</t>
         </is>
       </c>
       <c r="B461" s="4" t="s">
@@ -21505,7 +21511,7 @@
     <row r="463" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A463" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000296</t>
+          <t xml:space="preserve">296</t>
         </is>
       </c>
       <c r="B463" s="4" t="s">
@@ -21546,7 +21552,7 @@
     <row r="464" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A464" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000297</t>
+          <t xml:space="preserve">297</t>
         </is>
       </c>
       <c r="B464" s="4" t="s">
@@ -21587,7 +21593,7 @@
     <row r="465" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A465" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000298</t>
+          <t xml:space="preserve">298</t>
         </is>
       </c>
       <c r="B465" s="4" t="s">
@@ -21628,7 +21634,7 @@
     <row r="466" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A466" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000299</t>
+          <t xml:space="preserve">299</t>
         </is>
       </c>
       <c r="B466" s="4" t="s">
@@ -21671,7 +21677,7 @@
     <row r="467" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A467" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000300</t>
+          <t xml:space="preserve">300</t>
         </is>
       </c>
       <c r="B467" s="4" t="s">
@@ -21737,7 +21743,7 @@
     <row r="469" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A469" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000301</t>
+          <t xml:space="preserve">301</t>
         </is>
       </c>
       <c r="B469" s="4" t="s">
@@ -21778,7 +21784,7 @@
     <row r="470" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A470" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000302</t>
+          <t xml:space="preserve">302</t>
         </is>
       </c>
       <c r="B470" s="4" t="s">
@@ -21838,7 +21844,7 @@
     <row r="472" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A472" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000303</t>
+          <t xml:space="preserve">303</t>
         </is>
       </c>
       <c r="B472" s="4" t="s">
@@ -21879,7 +21885,7 @@
     <row r="473" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A473" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000304</t>
+          <t xml:space="preserve">304</t>
         </is>
       </c>
       <c r="B473" s="4" t="s">
@@ -21920,7 +21926,7 @@
     <row r="474" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A474" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000305</t>
+          <t xml:space="preserve">305</t>
         </is>
       </c>
       <c r="B474" s="4" t="s">
@@ -21961,7 +21967,7 @@
     <row r="475" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A475" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000306</t>
+          <t xml:space="preserve">306</t>
         </is>
       </c>
       <c r="B475" s="4" t="s">
@@ -22002,7 +22008,7 @@
     <row r="476" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A476" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000307</t>
+          <t xml:space="preserve">307</t>
         </is>
       </c>
       <c r="B476" s="4" t="s">
@@ -22041,7 +22047,7 @@
     <row r="477" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A477" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000308</t>
+          <t xml:space="preserve">308</t>
         </is>
       </c>
       <c r="B477" s="4" t="s">
@@ -22107,7 +22113,7 @@
     <row r="479" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A479" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000309</t>
+          <t xml:space="preserve">309</t>
         </is>
       </c>
       <c r="B479" s="4" t="s">
@@ -22148,7 +22154,7 @@
     <row r="480" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A480" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000310</t>
+          <t xml:space="preserve">310</t>
         </is>
       </c>
       <c r="B480" s="4" t="s">
@@ -22212,7 +22218,7 @@
     <row r="482" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A482" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000311</t>
+          <t xml:space="preserve">311</t>
         </is>
       </c>
       <c r="B482" s="4" t="s">
@@ -22253,7 +22259,7 @@
     <row r="483" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A483" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000312</t>
+          <t xml:space="preserve">312</t>
         </is>
       </c>
       <c r="B483" s="4" t="s">
@@ -22294,7 +22300,7 @@
     <row r="484" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A484" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000313</t>
+          <t xml:space="preserve">313</t>
         </is>
       </c>
       <c r="B484" s="4" t="s">
@@ -22335,7 +22341,7 @@
     <row r="485" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A485" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000314</t>
+          <t xml:space="preserve">314</t>
         </is>
       </c>
       <c r="B485" s="4" t="s">
@@ -22376,7 +22382,7 @@
     <row r="486" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A486" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000315</t>
+          <t xml:space="preserve">315</t>
         </is>
       </c>
       <c r="B486" s="4" t="s">
@@ -22417,7 +22423,7 @@
     <row r="487" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A487" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000316</t>
+          <t xml:space="preserve">316</t>
         </is>
       </c>
       <c r="B487" s="4" t="s">
@@ -22458,7 +22464,7 @@
     <row r="488" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A488" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000317</t>
+          <t xml:space="preserve">317</t>
         </is>
       </c>
       <c r="B488" s="4" t="s">
@@ -22499,7 +22505,7 @@
     <row r="489" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A489" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000318</t>
+          <t xml:space="preserve">318</t>
         </is>
       </c>
       <c r="B489" s="4" t="s">
@@ -22540,7 +22546,7 @@
     <row r="490" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A490" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000319</t>
+          <t xml:space="preserve">319</t>
         </is>
       </c>
       <c r="B490" s="4" t="s">
@@ -22575,7 +22581,7 @@
     <row r="491" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A491" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000320</t>
+          <t xml:space="preserve">320</t>
         </is>
       </c>
       <c r="B491" s="4" t="s">
@@ -22616,7 +22622,7 @@
     <row r="492" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A492" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000321</t>
+          <t xml:space="preserve">321</t>
         </is>
       </c>
       <c r="B492" s="4" t="s">
@@ -22657,7 +22663,7 @@
     <row r="493" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A493" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000322</t>
+          <t xml:space="preserve">322</t>
         </is>
       </c>
       <c r="B493" s="4" t="s">
@@ -22698,7 +22704,7 @@
     <row r="494" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A494" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000323</t>
+          <t xml:space="preserve">323</t>
         </is>
       </c>
       <c r="B494" s="4" t="s">
@@ -22739,7 +22745,7 @@
     <row r="495" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A495" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000324</t>
+          <t xml:space="preserve">324</t>
         </is>
       </c>
       <c r="B495" s="4" t="s">
@@ -22780,7 +22786,7 @@
     <row r="496" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A496" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000325</t>
+          <t xml:space="preserve">325</t>
         </is>
       </c>
       <c r="B496" s="4" t="s">
@@ -22821,7 +22827,7 @@
     <row r="497" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A497" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000326</t>
+          <t xml:space="preserve">326</t>
         </is>
       </c>
       <c r="B497" s="4" t="s">
@@ -22862,7 +22868,7 @@
     <row r="498" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A498" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000327</t>
+          <t xml:space="preserve">327</t>
         </is>
       </c>
       <c r="B498" s="4" t="s">
@@ -22903,7 +22909,7 @@
     <row r="499" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A499" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000328</t>
+          <t xml:space="preserve">328</t>
         </is>
       </c>
       <c r="B499" s="4" t="s">
@@ -22938,7 +22944,7 @@
     <row r="500" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A500" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000329</t>
+          <t xml:space="preserve">329</t>
         </is>
       </c>
       <c r="B500" s="4" t="s">
@@ -22979,7 +22985,7 @@
     <row r="501" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A501" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000330</t>
+          <t xml:space="preserve">330</t>
         </is>
       </c>
       <c r="B501" s="4" t="s">
@@ -23020,7 +23026,7 @@
     <row r="502" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A502" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000331</t>
+          <t xml:space="preserve">331</t>
         </is>
       </c>
       <c r="B502" s="4" t="s">
@@ -23061,7 +23067,7 @@
     <row r="503" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A503" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000332</t>
+          <t xml:space="preserve">332</t>
         </is>
       </c>
       <c r="B503" s="4" t="s">
@@ -23102,7 +23108,7 @@
     <row r="504" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A504" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000333</t>
+          <t xml:space="preserve">333</t>
         </is>
       </c>
       <c r="B504" s="4" t="s">
@@ -23166,7 +23172,7 @@
     <row r="506" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A506" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000334</t>
+          <t xml:space="preserve">334</t>
         </is>
       </c>
       <c r="B506" s="4" t="s">
@@ -23207,7 +23213,7 @@
     <row r="507" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A507" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000335</t>
+          <t xml:space="preserve">335</t>
         </is>
       </c>
       <c r="B507" s="4" t="s">
@@ -23248,7 +23254,7 @@
     <row r="508" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A508" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000336</t>
+          <t xml:space="preserve">336</t>
         </is>
       </c>
       <c r="B508" s="4" t="s">
@@ -23289,7 +23295,7 @@
     <row r="509" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A509" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000337</t>
+          <t xml:space="preserve">337</t>
         </is>
       </c>
       <c r="B509" s="4" t="s">
@@ -23330,7 +23336,7 @@
     <row r="510" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A510" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000338</t>
+          <t xml:space="preserve">338</t>
         </is>
       </c>
       <c r="B510" s="4" t="s">
@@ -23371,7 +23377,7 @@
     <row r="511" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A511" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000339</t>
+          <t xml:space="preserve">339</t>
         </is>
       </c>
       <c r="B511" s="4" t="s">
@@ -23412,7 +23418,7 @@
     <row r="512" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A512" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000340</t>
+          <t xml:space="preserve">340</t>
         </is>
       </c>
       <c r="B512" s="4" t="s">
@@ -23453,7 +23459,7 @@
     <row r="513" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A513" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000341</t>
+          <t xml:space="preserve">341</t>
         </is>
       </c>
       <c r="B513" s="4" t="s">
@@ -23494,7 +23500,7 @@
     <row r="514" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A514" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000342</t>
+          <t xml:space="preserve">342</t>
         </is>
       </c>
       <c r="B514" s="4" t="s">
@@ -23535,7 +23541,7 @@
     <row r="515" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A515" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000343</t>
+          <t xml:space="preserve">343</t>
         </is>
       </c>
       <c r="B515" s="4" t="s">
@@ -23576,7 +23582,7 @@
     <row r="516" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A516" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000344</t>
+          <t xml:space="preserve">344</t>
         </is>
       </c>
       <c r="B516" s="4" t="s">
@@ -23615,7 +23621,7 @@
     <row r="517" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A517" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000345</t>
+          <t xml:space="preserve">345</t>
         </is>
       </c>
       <c r="B517" s="4" t="s">
@@ -23656,7 +23662,7 @@
     <row r="518" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A518" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000346</t>
+          <t xml:space="preserve">346</t>
         </is>
       </c>
       <c r="B518" s="4" t="s">
@@ -23697,7 +23703,7 @@
     <row r="519" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A519" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000347</t>
+          <t xml:space="preserve">347</t>
         </is>
       </c>
       <c r="B519" s="4" t="s">
@@ -23763,7 +23769,7 @@
     <row r="521" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A521" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000348</t>
+          <t xml:space="preserve">348</t>
         </is>
       </c>
       <c r="B521" s="4" t="s">
@@ -23804,7 +23810,7 @@
     <row r="522" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A522" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000349</t>
+          <t xml:space="preserve">349</t>
         </is>
       </c>
       <c r="B522" s="4" t="s">
@@ -23845,7 +23851,7 @@
     <row r="523" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A523" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000350</t>
+          <t xml:space="preserve">350</t>
         </is>
       </c>
       <c r="B523" s="4" t="s">
@@ -23913,7 +23919,7 @@
     <row r="525" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A525" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000351</t>
+          <t xml:space="preserve">351</t>
         </is>
       </c>
       <c r="B525" s="4" t="s">
@@ -23979,7 +23985,7 @@
     <row r="527" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A527" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000352</t>
+          <t xml:space="preserve">352</t>
         </is>
       </c>
       <c r="B527" s="4" t="s">
@@ -24045,7 +24051,7 @@
     <row r="529" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A529" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000353</t>
+          <t xml:space="preserve">353</t>
         </is>
       </c>
       <c r="B529" s="4" t="s">
@@ -24111,7 +24117,7 @@
     <row r="531" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A531" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000354</t>
+          <t xml:space="preserve">354</t>
         </is>
       </c>
       <c r="B531" s="4" t="s">
@@ -24152,7 +24158,7 @@
     <row r="532" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A532" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000355</t>
+          <t xml:space="preserve">355</t>
         </is>
       </c>
       <c r="B532" s="4" t="s">
@@ -24193,7 +24199,7 @@
     <row r="533" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A533" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000356</t>
+          <t xml:space="preserve">356</t>
         </is>
       </c>
       <c r="B533" s="4" t="s">
@@ -24234,7 +24240,7 @@
     <row r="534" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A534" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000357</t>
+          <t xml:space="preserve">357</t>
         </is>
       </c>
       <c r="B534" s="4" t="s">
@@ -24275,7 +24281,7 @@
     <row r="535" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A535" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000358</t>
+          <t xml:space="preserve">358</t>
         </is>
       </c>
       <c r="B535" s="4" t="s">
@@ -24316,7 +24322,7 @@
     <row r="536" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A536" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000359</t>
+          <t xml:space="preserve">359</t>
         </is>
       </c>
       <c r="B536" s="4" t="s">
@@ -24357,7 +24363,7 @@
     <row r="537" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A537" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000360</t>
+          <t xml:space="preserve">360</t>
         </is>
       </c>
       <c r="B537" s="4" t="s">
@@ -24396,7 +24402,7 @@
     <row r="538" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A538" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000361</t>
+          <t xml:space="preserve">361</t>
         </is>
       </c>
       <c r="B538" s="4" t="s">
@@ -24437,7 +24443,7 @@
     <row r="539" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A539" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000362</t>
+          <t xml:space="preserve">362</t>
         </is>
       </c>
       <c r="B539" s="4" t="s">
@@ -24503,7 +24509,7 @@
     <row r="541" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A541" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000363</t>
+          <t xml:space="preserve">363</t>
         </is>
       </c>
       <c r="B541" s="4" t="s">
@@ -24565,7 +24571,7 @@
     <row r="543" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A543" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000364</t>
+          <t xml:space="preserve">364</t>
         </is>
       </c>
       <c r="B543" s="4" t="s">
@@ -24606,7 +24612,7 @@
     <row r="544" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A544" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000365</t>
+          <t xml:space="preserve">365</t>
         </is>
       </c>
       <c r="B544" s="4" t="s">
@@ -24647,7 +24653,7 @@
     <row r="545" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A545" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000366</t>
+          <t xml:space="preserve">366</t>
         </is>
       </c>
       <c r="B545" s="4" t="s">
@@ -24688,7 +24694,7 @@
     <row r="546" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A546" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000367</t>
+          <t xml:space="preserve">367</t>
         </is>
       </c>
       <c r="B546" s="4" t="s">
@@ -24729,7 +24735,7 @@
     <row r="547" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A547" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000368</t>
+          <t xml:space="preserve">368</t>
         </is>
       </c>
       <c r="B547" s="4" t="s">
@@ -24770,7 +24776,7 @@
     <row r="548" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A548" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000369</t>
+          <t xml:space="preserve">369</t>
         </is>
       </c>
       <c r="B548" s="4" t="s">
@@ -24811,7 +24817,7 @@
     <row r="549" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A549" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000370</t>
+          <t xml:space="preserve">370</t>
         </is>
       </c>
       <c r="B549" s="4" t="s">
@@ -24850,7 +24856,7 @@
     <row r="550" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A550" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000371</t>
+          <t xml:space="preserve">371</t>
         </is>
       </c>
       <c r="B550" s="4" t="s">
@@ -24916,7 +24922,7 @@
     <row r="552" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A552" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000372</t>
+          <t xml:space="preserve">372</t>
         </is>
       </c>
       <c r="B552" s="4" t="s">
@@ -24957,7 +24963,7 @@
     <row r="553" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A553" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000373</t>
+          <t xml:space="preserve">373</t>
         </is>
       </c>
       <c r="B553" s="4" t="s">
@@ -25048,7 +25054,7 @@
     <row r="556" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A556" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000374</t>
+          <t xml:space="preserve">374</t>
         </is>
       </c>
       <c r="B556" s="4" t="s">
@@ -25089,7 +25095,7 @@
     <row r="557" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A557" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000375</t>
+          <t xml:space="preserve">375</t>
         </is>
       </c>
       <c r="B557" s="4" t="s">
@@ -25130,7 +25136,7 @@
     <row r="558" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A558" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000376</t>
+          <t xml:space="preserve">376</t>
         </is>
       </c>
       <c r="B558" s="4" t="s">
@@ -25171,7 +25177,7 @@
     <row r="559" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A559" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000377</t>
+          <t xml:space="preserve">377</t>
         </is>
       </c>
       <c r="B559" s="4" t="s">
@@ -25237,7 +25243,7 @@
     <row r="561" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A561" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000378</t>
+          <t xml:space="preserve">378</t>
         </is>
       </c>
       <c r="B561" s="4" t="s">
@@ -25278,7 +25284,7 @@
     <row r="562" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A562" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000379</t>
+          <t xml:space="preserve">379</t>
         </is>
       </c>
       <c r="B562" s="4" t="s">
@@ -25321,7 +25327,7 @@
     <row r="563" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A563" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000380</t>
+          <t xml:space="preserve">380</t>
         </is>
       </c>
       <c r="B563" s="4" t="s">
@@ -25362,7 +25368,7 @@
     <row r="564" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A564" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000381</t>
+          <t xml:space="preserve">381</t>
         </is>
       </c>
       <c r="B564" s="4" t="s">
@@ -25403,7 +25409,7 @@
     <row r="565" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A565" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000382</t>
+          <t xml:space="preserve">382</t>
         </is>
       </c>
       <c r="B565" s="4" t="s">
@@ -25444,7 +25450,7 @@
     <row r="566" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A566" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000383</t>
+          <t xml:space="preserve">383</t>
         </is>
       </c>
       <c r="B566" s="4" t="s">
@@ -25485,7 +25491,7 @@
     <row r="567" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A567" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000384</t>
+          <t xml:space="preserve">384</t>
         </is>
       </c>
       <c r="B567" s="4" t="s">
@@ -25526,7 +25532,7 @@
     <row r="568" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A568" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000385</t>
+          <t xml:space="preserve">385</t>
         </is>
       </c>
       <c r="B568" s="4" t="s">
@@ -25565,7 +25571,7 @@
     <row r="569" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A569" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000386</t>
+          <t xml:space="preserve">386</t>
         </is>
       </c>
       <c r="B569" s="4" t="s">
@@ -25604,7 +25610,7 @@
     <row r="570" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A570" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000387</t>
+          <t xml:space="preserve">387</t>
         </is>
       </c>
       <c r="B570" s="4" t="s">
@@ -25643,7 +25649,7 @@
     <row r="571" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A571" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000388</t>
+          <t xml:space="preserve">388</t>
         </is>
       </c>
       <c r="B571" s="4" t="s">
@@ -25684,7 +25690,7 @@
     <row r="572" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A572" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000389</t>
+          <t xml:space="preserve">389</t>
         </is>
       </c>
       <c r="B572" s="4" t="s">
@@ -25725,7 +25731,7 @@
     <row r="573" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A573" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000390</t>
+          <t xml:space="preserve">390</t>
         </is>
       </c>
       <c r="B573" s="4" t="s">
@@ -25768,7 +25774,7 @@
     <row r="574" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A574" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000391</t>
+          <t xml:space="preserve">391</t>
         </is>
       </c>
       <c r="B574" s="4" t="s">
@@ -25809,7 +25815,7 @@
     <row r="575" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A575" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000392</t>
+          <t xml:space="preserve">392</t>
         </is>
       </c>
       <c r="B575" s="4" t="s">
@@ -25850,7 +25856,7 @@
     <row r="576" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A576" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000393</t>
+          <t xml:space="preserve">393</t>
         </is>
       </c>
       <c r="B576" s="4" t="s">
@@ -25891,7 +25897,7 @@
     <row r="577" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A577" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000394</t>
+          <t xml:space="preserve">394</t>
         </is>
       </c>
       <c r="B577" s="4" t="s">
@@ -25932,7 +25938,7 @@
     <row r="578" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A578" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000395</t>
+          <t xml:space="preserve">395</t>
         </is>
       </c>
       <c r="B578" s="4" t="s">
@@ -26010,7 +26016,7 @@
     <row r="580" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A580" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000396</t>
+          <t xml:space="preserve">396</t>
         </is>
       </c>
       <c r="B580" s="4" t="s">
@@ -26051,7 +26057,7 @@
     <row r="581" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A581" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000397</t>
+          <t xml:space="preserve">397</t>
         </is>
       </c>
       <c r="B581" s="4" t="s">
@@ -26086,7 +26092,7 @@
     <row r="582" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A582" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000398</t>
+          <t xml:space="preserve">398</t>
         </is>
       </c>
       <c r="B582" s="4" t="s">
@@ -26152,7 +26158,7 @@
     <row r="584" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A584" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000399</t>
+          <t xml:space="preserve">399</t>
         </is>
       </c>
       <c r="B584" s="4" t="s">
@@ -26193,7 +26199,7 @@
     <row r="585" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A585" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000400</t>
+          <t xml:space="preserve">400</t>
         </is>
       </c>
       <c r="B585" s="4" t="s">
@@ -26234,7 +26240,7 @@
     <row r="586" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A586" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000401</t>
+          <t xml:space="preserve">401</t>
         </is>
       </c>
       <c r="B586" s="4" t="s">
@@ -26275,7 +26281,7 @@
     <row r="587" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A587" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000402</t>
+          <t xml:space="preserve">402</t>
         </is>
       </c>
       <c r="B587" s="4" t="s">
@@ -26355,7 +26361,7 @@
     <row r="589" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A589" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000403</t>
+          <t xml:space="preserve">403</t>
         </is>
       </c>
       <c r="B589" s="4" t="s">
@@ -26396,7 +26402,7 @@
     <row r="590" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A590" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000404</t>
+          <t xml:space="preserve">404</t>
         </is>
       </c>
       <c r="B590" s="4" t="s">
@@ -26437,7 +26443,7 @@
     <row r="591" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A591" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000405</t>
+          <t xml:space="preserve">405</t>
         </is>
       </c>
       <c r="B591" s="4" t="s">
@@ -26478,7 +26484,7 @@
     <row r="592" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A592" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000406</t>
+          <t xml:space="preserve">406</t>
         </is>
       </c>
       <c r="B592" s="4" t="s">
@@ -26519,7 +26525,7 @@
     <row r="593" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A593" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000407</t>
+          <t xml:space="preserve">407</t>
         </is>
       </c>
       <c r="B593" s="4" t="s">
@@ -26562,7 +26568,7 @@
     <row r="594" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A594" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000408</t>
+          <t xml:space="preserve">408</t>
         </is>
       </c>
       <c r="B594" s="4" t="s">
@@ -26603,7 +26609,7 @@
     <row r="595" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A595" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000409</t>
+          <t xml:space="preserve">409</t>
         </is>
       </c>
       <c r="B595" s="4" t="s">
@@ -26644,7 +26650,7 @@
     <row r="596" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A596" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000410</t>
+          <t xml:space="preserve">410</t>
         </is>
       </c>
       <c r="B596" s="4" t="s">
@@ -26683,7 +26689,7 @@
     <row r="597" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A597" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000411</t>
+          <t xml:space="preserve">411</t>
         </is>
       </c>
       <c r="B597" s="4" t="s">
@@ -26724,7 +26730,7 @@
     <row r="598" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A598" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000412</t>
+          <t xml:space="preserve">412</t>
         </is>
       </c>
       <c r="B598" s="4" t="s">
@@ -26790,7 +26796,7 @@
     <row r="600" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A600" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000413</t>
+          <t xml:space="preserve">413</t>
         </is>
       </c>
       <c r="B600" s="4" t="s">
@@ -26831,7 +26837,7 @@
     <row r="601" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A601" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000414</t>
+          <t xml:space="preserve">414</t>
         </is>
       </c>
       <c r="B601" s="4" t="s">
@@ -26872,7 +26878,7 @@
     <row r="602" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A602" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000415</t>
+          <t xml:space="preserve">415</t>
         </is>
       </c>
       <c r="B602" s="4" t="s">
@@ -26936,7 +26942,7 @@
     <row r="604" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A604" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000416</t>
+          <t xml:space="preserve">416</t>
         </is>
       </c>
       <c r="B604" s="4" t="s">
@@ -26977,7 +26983,7 @@
     <row r="605" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A605" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000417</t>
+          <t xml:space="preserve">417</t>
         </is>
       </c>
       <c r="B605" s="4" t="s">
@@ -27016,7 +27022,7 @@
     <row r="606" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A606" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000418</t>
+          <t xml:space="preserve">418</t>
         </is>
       </c>
       <c r="B606" s="4" t="s">
@@ -27057,7 +27063,7 @@
     <row r="607" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A607" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000419</t>
+          <t xml:space="preserve">419</t>
         </is>
       </c>
       <c r="B607" s="4" t="s">
@@ -27098,7 +27104,7 @@
     <row r="608" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A608" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000420</t>
+          <t xml:space="preserve">420</t>
         </is>
       </c>
       <c r="B608" s="4" t="s">
@@ -27139,7 +27145,7 @@
     <row r="609" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A609" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000421</t>
+          <t xml:space="preserve">421</t>
         </is>
       </c>
       <c r="B609" s="4" t="s">
@@ -27180,7 +27186,7 @@
     <row r="610" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A610" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000422</t>
+          <t xml:space="preserve">422</t>
         </is>
       </c>
       <c r="B610" s="4" t="s">
@@ -27221,7 +27227,7 @@
     <row r="611" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A611" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000423</t>
+          <t xml:space="preserve">423</t>
         </is>
       </c>
       <c r="B611" s="4" t="s">
@@ -27262,7 +27268,7 @@
     <row r="612" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A612" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000424</t>
+          <t xml:space="preserve">424</t>
         </is>
       </c>
       <c r="B612" s="4" t="s">
@@ -27299,7 +27305,7 @@
     <row r="613" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A613" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000425</t>
+          <t xml:space="preserve">425</t>
         </is>
       </c>
       <c r="B613" s="4" t="s">
@@ -27390,7 +27396,7 @@
     <row r="616" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A616" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000426</t>
+          <t xml:space="preserve">426</t>
         </is>
       </c>
       <c r="B616" s="4" t="s">
@@ -27431,7 +27437,7 @@
     <row r="617" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A617" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000427</t>
+          <t xml:space="preserve">427</t>
         </is>
       </c>
       <c r="B617" s="4" t="s">
@@ -27472,7 +27478,7 @@
     <row r="618" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A618" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000428</t>
+          <t xml:space="preserve">428</t>
         </is>
       </c>
       <c r="B618" s="4" t="s">
@@ -27509,7 +27515,7 @@
     <row r="619" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A619" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000429</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B619" s="4" t="s">
@@ -27548,7 +27554,7 @@
     <row r="620" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A620" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000430</t>
+          <t xml:space="preserve">430</t>
         </is>
       </c>
       <c r="B620" s="4" t="s">
@@ -27589,7 +27595,7 @@
     <row r="621" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A621" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000431</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B621" s="4" t="s">
@@ -27630,7 +27636,7 @@
     <row r="622" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A622" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000432</t>
+          <t xml:space="preserve">432</t>
         </is>
       </c>
       <c r="B622" s="4" t="s">
@@ -27696,7 +27702,7 @@
     <row r="624" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A624" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000433</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B624" s="4" t="s">
@@ -27737,7 +27743,7 @@
     <row r="625" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A625" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000434</t>
+          <t xml:space="preserve">434</t>
         </is>
       </c>
       <c r="B625" s="4" t="s">
@@ -27776,7 +27782,7 @@
     <row r="626" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A626" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000435</t>
+          <t xml:space="preserve">435</t>
         </is>
       </c>
       <c r="B626" s="4" t="s">
@@ -27867,7 +27873,7 @@
     <row r="629" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A629" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000436</t>
+          <t xml:space="preserve">436</t>
         </is>
       </c>
       <c r="B629" s="4" t="s">
@@ -27908,7 +27914,7 @@
     <row r="630" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A630" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000437</t>
+          <t xml:space="preserve">437</t>
         </is>
       </c>
       <c r="B630" s="4" t="s">
@@ -27949,7 +27955,7 @@
     <row r="631" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A631" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000438</t>
+          <t xml:space="preserve">438</t>
         </is>
       </c>
       <c r="B631" s="4" t="s">
@@ -27988,7 +27994,7 @@
     <row r="632" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A632" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000439</t>
+          <t xml:space="preserve">439</t>
         </is>
       </c>
       <c r="B632" s="4" t="s">
@@ -28023,7 +28029,7 @@
     <row r="633" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A633" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000440</t>
+          <t xml:space="preserve">440</t>
         </is>
       </c>
       <c r="B633" s="4" t="s">
@@ -28087,7 +28093,7 @@
     <row r="635" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A635" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000441</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B635" s="4" t="s">
@@ -28128,7 +28134,7 @@
     <row r="636" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A636" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000442</t>
+          <t xml:space="preserve">442</t>
         </is>
       </c>
       <c r="B636" s="4" t="s">
@@ -28194,7 +28200,7 @@
     <row r="638" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A638" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000443</t>
+          <t xml:space="preserve">443</t>
         </is>
       </c>
       <c r="B638" s="4" t="s">
@@ -28237,7 +28243,7 @@
     <row r="639" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A639" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000444</t>
+          <t xml:space="preserve">444</t>
         </is>
       </c>
       <c r="B639" s="4" t="s">
@@ -28276,7 +28282,7 @@
     <row r="640" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A640" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000445</t>
+          <t xml:space="preserve">445</t>
         </is>
       </c>
       <c r="B640" s="4" t="s">
@@ -28317,7 +28323,7 @@
     <row r="641" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A641" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000446</t>
+          <t xml:space="preserve">446</t>
         </is>
       </c>
       <c r="B641" s="4" t="s">
@@ -28358,7 +28364,7 @@
     <row r="642" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A642" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000447</t>
+          <t xml:space="preserve">447</t>
         </is>
       </c>
       <c r="B642" s="4" t="s">
@@ -28397,7 +28403,7 @@
     <row r="643" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A643" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000448</t>
+          <t xml:space="preserve">448</t>
         </is>
       </c>
       <c r="B643" s="4" t="s">
@@ -28438,7 +28444,7 @@
     <row r="644" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A644" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000449</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B644" s="4" t="s">
@@ -28527,7 +28533,7 @@
     <row r="647" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A647" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000450</t>
+          <t xml:space="preserve">450</t>
         </is>
       </c>
       <c r="B647" s="4" t="s">
@@ -28568,7 +28574,7 @@
     <row r="648" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A648" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000451</t>
+          <t xml:space="preserve">451</t>
         </is>
       </c>
       <c r="B648" s="4" t="s">
@@ -28609,7 +28615,7 @@
     <row r="649" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A649" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000452</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B649" s="4" t="s">
@@ -28675,7 +28681,7 @@
     <row r="651" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A651" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000453</t>
+          <t xml:space="preserve">453</t>
         </is>
       </c>
       <c r="B651" s="4" t="s">
@@ -28716,7 +28722,7 @@
     <row r="652" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A652" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000454</t>
+          <t xml:space="preserve">454</t>
         </is>
       </c>
       <c r="B652" s="4" t="s">
@@ -28751,7 +28757,7 @@
     <row r="653" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A653" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000455</t>
+          <t xml:space="preserve">455</t>
         </is>
       </c>
       <c r="B653" s="4" t="s">
@@ -28786,7 +28792,7 @@
     <row r="654" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A654" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000456</t>
+          <t xml:space="preserve">456</t>
         </is>
       </c>
       <c r="B654" s="4" t="s">
@@ -28827,7 +28833,7 @@
     <row r="655" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A655" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000457</t>
+          <t xml:space="preserve">457</t>
         </is>
       </c>
       <c r="B655" s="4" t="s">
@@ -28993,7 +28999,7 @@
     <row r="661" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A661" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000458</t>
+          <t xml:space="preserve">458</t>
         </is>
       </c>
       <c r="B661" s="4" t="s">
@@ -29034,7 +29040,7 @@
     <row r="662" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A662" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000459</t>
+          <t xml:space="preserve">459</t>
         </is>
       </c>
       <c r="B662" s="4" t="s">
@@ -29069,7 +29075,7 @@
     <row r="663" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A663" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000460</t>
+          <t xml:space="preserve">460</t>
         </is>
       </c>
       <c r="B663" s="4" t="s">
@@ -29110,7 +29116,7 @@
     <row r="664" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A664" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000461</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B664" s="4" t="s">
@@ -29176,7 +29182,7 @@
     <row r="666" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A666" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000462</t>
+          <t xml:space="preserve">462</t>
         </is>
       </c>
       <c r="B666" s="4" t="s">
@@ -29217,7 +29223,7 @@
     <row r="667" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A667" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000463</t>
+          <t xml:space="preserve">463</t>
         </is>
       </c>
       <c r="B667" s="4" t="s">
@@ -29258,7 +29264,7 @@
     <row r="668" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A668" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000464</t>
+          <t xml:space="preserve">464</t>
         </is>
       </c>
       <c r="B668" s="4" t="s">
@@ -29299,7 +29305,7 @@
     <row r="669" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A669" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000465</t>
+          <t xml:space="preserve">465</t>
         </is>
       </c>
       <c r="B669" s="4" t="s">
@@ -29340,7 +29346,7 @@
     <row r="670" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A670" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000466</t>
+          <t xml:space="preserve">466</t>
         </is>
       </c>
       <c r="B670" s="4" t="s">
@@ -40839,7 +40845,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-17 19:09</t>
+          <t xml:space="preserve">2026-10-18 18:27</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -40849,12 +40855,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000467</t>
+          <t xml:space="preserve">467</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">T.01102736</t>
+          <t xml:space="preserve">T.01104116</t>
         </is>
       </c>
       <c r="E2">
@@ -40869,7 +40875,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-17 19:11</t>
+          <t xml:space="preserve">2026-10-18 18:28</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -40879,16 +40885,16 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000467</t>
+          <t xml:space="preserve">467</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">T.01102736</t>
+          <t xml:space="preserve">T.01104116</t>
         </is>
       </c>
       <c r="E3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -40904,7 +40910,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-17 19:12</t>
+          <t xml:space="preserve">2026-10-18 18:29</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -40914,16 +40920,16 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAR-000467</t>
+          <t xml:space="preserve">467</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">T.01102736</t>
+          <t xml:space="preserve">T.01104116</t>
         </is>
       </c>
       <c r="E4">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -40933,106 +40939,6 @@
       <c r="H4" t="inlineStr">
         <is>
           <t xml:space="preserve">Retiro de tarima completa</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-10-17 19:13</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RECIBO</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAR-000467</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T.01107263</t>
-        </is>
-      </c>
-      <c r="E5">
-        <v>2</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R01-03B-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-10-17 19:14</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SURTIDO</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAR-000467</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T.01107263</t>
-        </is>
-      </c>
-      <c r="E6">
-        <v>-1</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R01-03B-02</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Retiro parcial de piezas</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-10-17 19:16</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SURTIDO</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAR-000467</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T.01107263</t>
-        </is>
-      </c>
-      <c r="E7">
-        <v>-1</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R01-03B-02</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Retiro parcial de piezas</t>
         </is>
       </c>
     </row>

</xml_diff>